<commit_message>
fix(lotte): preserve vehicle records by work shift
</commit_message>
<xml_diff>
--- a/home/src/site_apps/lotte/data/Lotte_Material_Inventory.xlsx
+++ b/home/src/site_apps/lotte/data/Lotte_Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,9 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,9 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24649,7 +24652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W140"/>
+  <dimension ref="A1:W150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32886,6 +32889,508 @@
       <c r="V140" t="inlineStr"/>
       <c r="W140" t="inlineStr"/>
     </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>46072.35869387732</v>
+      </c>
+      <c r="B141" t="n">
+        <v>420</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>부장 주진철, 부장 이봉주</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
+      <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr"/>
+      <c r="T141" t="inlineStr"/>
+      <c r="U141" t="inlineStr"/>
+      <c r="V141" t="inlineStr"/>
+      <c r="W141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>46072.35869387732</v>
+      </c>
+      <c r="B142" t="n">
+        <v>418</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>부장 주진철, 부장 이봉주</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr"/>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="inlineStr"/>
+      <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
+      <c r="P142" t="inlineStr"/>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr"/>
+      <c r="T142" t="inlineStr"/>
+      <c r="U142" t="inlineStr"/>
+      <c r="V142" t="inlineStr"/>
+      <c r="W142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B143" t="n">
+        <v>410</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>-42</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>주임 김성렬, 대리 우명광</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="inlineStr"/>
+      <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
+      <c r="P143" t="inlineStr"/>
+      <c r="Q143" t="inlineStr"/>
+      <c r="R143" t="inlineStr"/>
+      <c r="S143" t="inlineStr"/>
+      <c r="T143" t="inlineStr"/>
+      <c r="U143" t="inlineStr"/>
+      <c r="V143" t="inlineStr"/>
+      <c r="W143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B144" t="n">
+        <v>410</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>-30</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>주임 김성렬, 대리 우명광</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr"/>
+      <c r="M144" t="inlineStr"/>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="inlineStr"/>
+      <c r="S144" t="inlineStr"/>
+      <c r="T144" t="inlineStr"/>
+      <c r="U144" t="inlineStr"/>
+      <c r="V144" t="inlineStr"/>
+      <c r="W144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>46078.38191709491</v>
+      </c>
+      <c r="B145" t="n">
+        <v>418</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>주임 박상태</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
+      <c r="P145" t="inlineStr"/>
+      <c r="Q145" t="inlineStr"/>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr"/>
+      <c r="T145" t="inlineStr"/>
+      <c r="U145" t="inlineStr"/>
+      <c r="V145" t="inlineStr"/>
+      <c r="W145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>46080.40617881263</v>
+      </c>
+      <c r="B146" t="n">
+        <v>420</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>부장 주진철, 주임 김진환</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
+      <c r="P146" t="inlineStr"/>
+      <c r="Q146" t="inlineStr"/>
+      <c r="R146" t="inlineStr"/>
+      <c r="S146" t="inlineStr"/>
+      <c r="T146" t="inlineStr"/>
+      <c r="U146" t="inlineStr"/>
+      <c r="V146" t="inlineStr"/>
+      <c r="W146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>46080.40617881263</v>
+      </c>
+      <c r="B147" t="n">
+        <v>418</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>부장 주진철, 주임 김진환</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr"/>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr"/>
+      <c r="T147" t="inlineStr"/>
+      <c r="U147" t="inlineStr"/>
+      <c r="V147" t="inlineStr"/>
+      <c r="W147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B148" t="n">
+        <v>410</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>-18</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>주임 김성렬, 대리 우명광, 부장 주진철</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="inlineStr"/>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
+      <c r="P148" t="inlineStr"/>
+      <c r="Q148" t="inlineStr"/>
+      <c r="R148" t="inlineStr"/>
+      <c r="S148" t="inlineStr"/>
+      <c r="T148" t="inlineStr"/>
+      <c r="U148" t="inlineStr"/>
+      <c r="V148" t="inlineStr"/>
+      <c r="W148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>46112.43436334715</v>
+      </c>
+      <c r="B149" t="n">
+        <v>420</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="inlineStr"/>
+      <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
+      <c r="P149" t="inlineStr"/>
+      <c r="Q149" t="inlineStr"/>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr"/>
+      <c r="T149" t="inlineStr"/>
+      <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr"/>
+      <c r="W149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B150" t="n">
+        <v>410</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>-15</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>K1 PJT 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>대리 김성현, 주임 김성렬, 주임 이경재</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
+      <c r="M150" t="inlineStr"/>
+      <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr"/>
+      <c r="P150" t="inlineStr"/>
+      <c r="Q150" t="inlineStr"/>
+      <c r="R150" t="inlineStr"/>
+      <c r="S150" t="inlineStr"/>
+      <c r="T150" t="inlineStr"/>
+      <c r="U150" t="inlineStr"/>
+      <c r="V150" t="inlineStr"/>
+      <c r="W150" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -32948,7 +33453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE159"/>
+  <dimension ref="A1:DE173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75792,6 +76297,3584 @@
         <v>0</v>
       </c>
     </row>
+    <row r="160">
+      <c r="A160" s="1" t="n">
+        <v>46072</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="n">
+        <v>50</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F160" s="1" t="n">
+        <v>46293.35869385417</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" t="n">
+        <v>0</v>
+      </c>
+      <c r="K160" t="n">
+        <v>0</v>
+      </c>
+      <c r="L160" t="n">
+        <v>0</v>
+      </c>
+      <c r="M160" t="n">
+        <v>0</v>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr"/>
+      <c r="P160" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>4200</v>
+      </c>
+      <c r="R160" t="n">
+        <v>0</v>
+      </c>
+      <c r="S160" t="n">
+        <v>0</v>
+      </c>
+      <c r="T160" t="n">
+        <v>210000</v>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="V160" t="n">
+        <v>0</v>
+      </c>
+      <c r="W160" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X160" t="inlineStr"/>
+      <c r="Y160" t="inlineStr">
+        <is>
+          <t>부장 이봉주</t>
+        </is>
+      </c>
+      <c r="Z160" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA160" t="inlineStr"/>
+      <c r="AB160" t="inlineStr"/>
+      <c r="AC160" t="inlineStr"/>
+      <c r="AD160" t="inlineStr"/>
+      <c r="AE160" t="inlineStr"/>
+      <c r="AF160" t="inlineStr"/>
+      <c r="AG160" t="inlineStr"/>
+      <c r="AH160" t="inlineStr"/>
+      <c r="AI160" t="inlineStr"/>
+      <c r="AJ160" t="inlineStr"/>
+      <c r="AK160" t="inlineStr"/>
+      <c r="AL160" t="inlineStr"/>
+      <c r="AM160" t="inlineStr"/>
+      <c r="AN160" t="inlineStr"/>
+      <c r="AO160" t="inlineStr"/>
+      <c r="AP160" t="inlineStr"/>
+      <c r="AQ160" t="inlineStr"/>
+      <c r="AR160" t="inlineStr"/>
+      <c r="AS160" t="inlineStr"/>
+      <c r="AT160" t="inlineStr"/>
+      <c r="AU160" t="inlineStr"/>
+      <c r="AV160" t="inlineStr"/>
+      <c r="AW160" t="inlineStr"/>
+      <c r="AX160" t="inlineStr"/>
+      <c r="AY160" t="inlineStr"/>
+      <c r="AZ160" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA160" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB160" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC160" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD160" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE160" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF160" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG160" t="inlineStr">
+        <is>
+          <t>81루5100 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH160" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="BI160" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ160" t="inlineStr"/>
+      <c r="BK160" t="inlineStr"/>
+      <c r="BL160" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM160" t="inlineStr"/>
+      <c r="BN160" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO160" t="inlineStr"/>
+      <c r="BP160" t="inlineStr"/>
+      <c r="BQ160" t="inlineStr"/>
+      <c r="BR160" t="inlineStr"/>
+      <c r="BS160" t="inlineStr"/>
+      <c r="BT160" t="inlineStr"/>
+      <c r="BU160" t="inlineStr"/>
+      <c r="BV160" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW160" t="inlineStr"/>
+      <c r="BX160" t="inlineStr"/>
+      <c r="BY160" t="inlineStr"/>
+      <c r="BZ160" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA160" t="inlineStr"/>
+      <c r="CB160" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC160" t="inlineStr">
+        <is>
+          <t>250mm 초과 [10인치 이상] (1.0)</t>
+        </is>
+      </c>
+      <c r="CD160" t="inlineStr"/>
+      <c r="CE160" t="inlineStr"/>
+      <c r="CF160" t="inlineStr"/>
+      <c r="CG160" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH160" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI160" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ160" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK160" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL160" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM160" t="inlineStr"/>
+      <c r="CN160" t="inlineStr"/>
+      <c r="CO160" t="inlineStr"/>
+      <c r="CP160" t="inlineStr"/>
+      <c r="CQ160" t="inlineStr"/>
+      <c r="CR160" t="inlineStr"/>
+      <c r="CS160" t="inlineStr"/>
+      <c r="CT160" t="inlineStr"/>
+      <c r="CU160" t="inlineStr"/>
+      <c r="CV160" t="inlineStr"/>
+      <c r="CW160" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX160" t="inlineStr"/>
+      <c r="CY160" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ160" t="inlineStr"/>
+      <c r="DA160" t="inlineStr"/>
+      <c r="DB160" t="inlineStr"/>
+      <c r="DC160" t="inlineStr"/>
+      <c r="DD160" t="inlineStr"/>
+      <c r="DE160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>410</v>
+      </c>
+      <c r="D161" t="n">
+        <v>42</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F161" s="1" t="n">
+        <v>46293.36184457176</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" t="n">
+        <v>0</v>
+      </c>
+      <c r="K161" t="n">
+        <v>0</v>
+      </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" t="n">
+        <v>0</v>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>주임 김성렬</t>
+        </is>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>R-ray(se-75)</t>
+        </is>
+      </c>
+      <c r="P161" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R161" t="n">
+        <v>0</v>
+      </c>
+      <c r="S161" t="n">
+        <v>0</v>
+      </c>
+      <c r="T161" t="n">
+        <v>1071000</v>
+      </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V161" t="n">
+        <v>0</v>
+      </c>
+      <c r="W161" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="X161" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="Y161" t="inlineStr">
+        <is>
+          <t>대리 우명광</t>
+        </is>
+      </c>
+      <c r="Z161" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="AA161" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="AB161" t="inlineStr"/>
+      <c r="AC161" t="inlineStr"/>
+      <c r="AD161" t="inlineStr"/>
+      <c r="AE161" t="inlineStr"/>
+      <c r="AF161" t="inlineStr"/>
+      <c r="AG161" t="inlineStr"/>
+      <c r="AH161" t="inlineStr"/>
+      <c r="AI161" t="inlineStr"/>
+      <c r="AJ161" t="inlineStr"/>
+      <c r="AK161" t="inlineStr"/>
+      <c r="AL161" t="inlineStr"/>
+      <c r="AM161" t="inlineStr"/>
+      <c r="AN161" t="inlineStr"/>
+      <c r="AO161" t="inlineStr"/>
+      <c r="AP161" t="inlineStr"/>
+      <c r="AQ161" t="inlineStr"/>
+      <c r="AR161" t="inlineStr"/>
+      <c r="AS161" t="inlineStr"/>
+      <c r="AT161" t="inlineStr"/>
+      <c r="AU161" t="inlineStr"/>
+      <c r="AV161" t="inlineStr"/>
+      <c r="AW161" t="inlineStr"/>
+      <c r="AX161" t="inlineStr"/>
+      <c r="AY161" t="inlineStr"/>
+      <c r="AZ161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG161" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH161" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI161" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="BJ161" t="inlineStr"/>
+      <c r="BK161" t="inlineStr"/>
+      <c r="BL161" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM161" t="inlineStr"/>
+      <c r="BN161" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO161" t="inlineStr"/>
+      <c r="BP161" t="inlineStr"/>
+      <c r="BQ161" t="inlineStr"/>
+      <c r="BR161" t="inlineStr"/>
+      <c r="BS161" t="inlineStr"/>
+      <c r="BT161" t="inlineStr"/>
+      <c r="BU161" t="inlineStr"/>
+      <c r="BV161" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW161" t="inlineStr"/>
+      <c r="BX161" t="inlineStr"/>
+      <c r="BY161" t="inlineStr"/>
+      <c r="BZ161" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA161" t="inlineStr"/>
+      <c r="CB161" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC161" t="inlineStr">
+        <is>
+          <t>Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD161" t="inlineStr">
+        <is>
+          <t>조건없음 (1.0)</t>
+        </is>
+      </c>
+      <c r="CE161" t="inlineStr"/>
+      <c r="CF161" t="inlineStr"/>
+      <c r="CG161" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH161" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI161" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ161" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK161" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL161" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM161" t="inlineStr"/>
+      <c r="CN161" t="inlineStr"/>
+      <c r="CO161" t="inlineStr"/>
+      <c r="CP161" t="inlineStr"/>
+      <c r="CQ161" t="inlineStr"/>
+      <c r="CR161" t="inlineStr"/>
+      <c r="CS161" t="inlineStr"/>
+      <c r="CT161" t="inlineStr"/>
+      <c r="CU161" t="inlineStr"/>
+      <c r="CV161" t="inlineStr"/>
+      <c r="CW161" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX161" t="inlineStr"/>
+      <c r="CY161" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ161" t="inlineStr"/>
+      <c r="DA161" t="inlineStr">
+        <is>
+          <t>주배관</t>
+        </is>
+      </c>
+      <c r="DB161" t="inlineStr"/>
+      <c r="DC161" t="inlineStr"/>
+      <c r="DD161" t="inlineStr"/>
+      <c r="DE161" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="n">
+        <v>90</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F162" s="1" t="n">
+        <v>46293.36334530092</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="n">
+        <v>0</v>
+      </c>
+      <c r="I162" t="n">
+        <v>0</v>
+      </c>
+      <c r="J162" t="n">
+        <v>0</v>
+      </c>
+      <c r="K162" t="n">
+        <v>0</v>
+      </c>
+      <c r="L162" t="n">
+        <v>0</v>
+      </c>
+      <c r="M162" t="n">
+        <v>0</v>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr"/>
+      <c r="P162" t="n">
+        <v>90</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>4200</v>
+      </c>
+      <c r="R162" t="n">
+        <v>0</v>
+      </c>
+      <c r="S162" t="n">
+        <v>0</v>
+      </c>
+      <c r="T162" t="n">
+        <v>378000</v>
+      </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="V162" t="n">
+        <v>0</v>
+      </c>
+      <c r="W162" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X162" t="inlineStr"/>
+      <c r="Y162" t="inlineStr">
+        <is>
+          <t>과장 유상훈</t>
+        </is>
+      </c>
+      <c r="Z162" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA162" t="inlineStr"/>
+      <c r="AB162" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="AC162" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AD162" t="inlineStr"/>
+      <c r="AE162" t="inlineStr">
+        <is>
+          <t>주임 이경재</t>
+        </is>
+      </c>
+      <c r="AF162" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AG162" t="inlineStr"/>
+      <c r="AH162" t="inlineStr"/>
+      <c r="AI162" t="inlineStr"/>
+      <c r="AJ162" t="inlineStr"/>
+      <c r="AK162" t="inlineStr"/>
+      <c r="AL162" t="inlineStr"/>
+      <c r="AM162" t="inlineStr"/>
+      <c r="AN162" t="inlineStr"/>
+      <c r="AO162" t="inlineStr"/>
+      <c r="AP162" t="inlineStr"/>
+      <c r="AQ162" t="inlineStr"/>
+      <c r="AR162" t="inlineStr"/>
+      <c r="AS162" t="inlineStr"/>
+      <c r="AT162" t="inlineStr"/>
+      <c r="AU162" t="inlineStr"/>
+      <c r="AV162" t="inlineStr"/>
+      <c r="AW162" t="inlineStr"/>
+      <c r="AX162" t="inlineStr"/>
+      <c r="AY162" t="inlineStr"/>
+      <c r="AZ162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG162" t="inlineStr">
+        <is>
+          <t>81루5100 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH162" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI162" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ162" t="inlineStr"/>
+      <c r="BK162" t="inlineStr"/>
+      <c r="BL162" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM162" t="inlineStr"/>
+      <c r="BN162" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO162" t="inlineStr"/>
+      <c r="BP162" t="inlineStr"/>
+      <c r="BQ162" t="inlineStr"/>
+      <c r="BR162" t="inlineStr"/>
+      <c r="BS162" t="inlineStr"/>
+      <c r="BT162" t="inlineStr"/>
+      <c r="BU162" t="inlineStr"/>
+      <c r="BV162" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW162" t="inlineStr"/>
+      <c r="BX162" t="inlineStr"/>
+      <c r="BY162" t="inlineStr"/>
+      <c r="BZ162" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA162" t="inlineStr"/>
+      <c r="CB162" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC162" t="inlineStr">
+        <is>
+          <t>250mm 초과 [10인치 이상] (1.0)</t>
+        </is>
+      </c>
+      <c r="CD162" t="inlineStr"/>
+      <c r="CE162" t="inlineStr"/>
+      <c r="CF162" t="inlineStr"/>
+      <c r="CG162" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH162" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI162" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ162" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK162" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL162" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM162" t="inlineStr"/>
+      <c r="CN162" t="inlineStr"/>
+      <c r="CO162" t="inlineStr"/>
+      <c r="CP162" t="inlineStr"/>
+      <c r="CQ162" t="inlineStr"/>
+      <c r="CR162" t="inlineStr"/>
+      <c r="CS162" t="inlineStr"/>
+      <c r="CT162" t="inlineStr"/>
+      <c r="CU162" t="inlineStr"/>
+      <c r="CV162" t="inlineStr"/>
+      <c r="CW162" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX162" t="inlineStr"/>
+      <c r="CY162" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ162" t="inlineStr"/>
+      <c r="DA162" t="inlineStr"/>
+      <c r="DB162" t="inlineStr"/>
+      <c r="DC162" t="inlineStr"/>
+      <c r="DD162" t="inlineStr"/>
+      <c r="DE162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>410</v>
+      </c>
+      <c r="D163" t="n">
+        <v>57</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F163" s="1" t="n">
+        <v>46293.3657733912</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="n">
+        <v>0</v>
+      </c>
+      <c r="I163" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" t="n">
+        <v>0</v>
+      </c>
+      <c r="K163" t="n">
+        <v>0</v>
+      </c>
+      <c r="L163" t="n">
+        <v>0</v>
+      </c>
+      <c r="M163" t="n">
+        <v>0</v>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>주임 김성렬</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>R-ray(se-75)</t>
+        </is>
+      </c>
+      <c r="P163" t="n">
+        <v>57</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R163" t="n">
+        <v>0</v>
+      </c>
+      <c r="S163" t="n">
+        <v>0</v>
+      </c>
+      <c r="T163" t="n">
+        <v>1453500</v>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V163" t="n">
+        <v>0</v>
+      </c>
+      <c r="W163" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="X163" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="Y163" t="inlineStr">
+        <is>
+          <t>대리 우명광</t>
+        </is>
+      </c>
+      <c r="Z163" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="AA163" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="AB163" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="AC163" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="AD163" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="AE163" t="inlineStr">
+        <is>
+          <t>주임 김성렬</t>
+        </is>
+      </c>
+      <c r="AF163" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="AG163" t="inlineStr"/>
+      <c r="AH163" t="inlineStr"/>
+      <c r="AI163" t="inlineStr"/>
+      <c r="AJ163" t="inlineStr"/>
+      <c r="AK163" t="inlineStr"/>
+      <c r="AL163" t="inlineStr"/>
+      <c r="AM163" t="inlineStr"/>
+      <c r="AN163" t="inlineStr"/>
+      <c r="AO163" t="inlineStr"/>
+      <c r="AP163" t="inlineStr"/>
+      <c r="AQ163" t="inlineStr"/>
+      <c r="AR163" t="inlineStr"/>
+      <c r="AS163" t="inlineStr"/>
+      <c r="AT163" t="inlineStr"/>
+      <c r="AU163" t="inlineStr"/>
+      <c r="AV163" t="inlineStr"/>
+      <c r="AW163" t="inlineStr"/>
+      <c r="AX163" t="inlineStr"/>
+      <c r="AY163" t="inlineStr"/>
+      <c r="AZ163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG163" t="inlineStr">
+        <is>
+          <t>81루5100 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH163" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI163" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="BJ163" t="inlineStr"/>
+      <c r="BK163" t="inlineStr"/>
+      <c r="BL163" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM163" t="inlineStr"/>
+      <c r="BN163" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO163" t="inlineStr"/>
+      <c r="BP163" t="inlineStr"/>
+      <c r="BQ163" t="inlineStr"/>
+      <c r="BR163" t="inlineStr"/>
+      <c r="BS163" t="inlineStr"/>
+      <c r="BT163" t="inlineStr"/>
+      <c r="BU163" t="inlineStr"/>
+      <c r="BV163" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW163" t="inlineStr"/>
+      <c r="BX163" t="inlineStr"/>
+      <c r="BY163" t="inlineStr"/>
+      <c r="BZ163" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA163" t="inlineStr"/>
+      <c r="CB163" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC163" t="inlineStr">
+        <is>
+          <t>Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD163" t="inlineStr">
+        <is>
+          <t>조건없음 (1.0)</t>
+        </is>
+      </c>
+      <c r="CE163" t="inlineStr"/>
+      <c r="CF163" t="inlineStr"/>
+      <c r="CG163" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH163" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI163" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ163" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK163" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL163" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM163" t="inlineStr"/>
+      <c r="CN163" t="inlineStr"/>
+      <c r="CO163" t="inlineStr"/>
+      <c r="CP163" t="inlineStr"/>
+      <c r="CQ163" t="inlineStr"/>
+      <c r="CR163" t="inlineStr"/>
+      <c r="CS163" t="inlineStr"/>
+      <c r="CT163" t="inlineStr"/>
+      <c r="CU163" t="inlineStr"/>
+      <c r="CV163" t="inlineStr"/>
+      <c r="CW163" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX163" t="inlineStr"/>
+      <c r="CY163" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ163" t="inlineStr"/>
+      <c r="DA163" t="inlineStr">
+        <is>
+          <t>주배관</t>
+        </is>
+      </c>
+      <c r="DB163" t="inlineStr"/>
+      <c r="DC163" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD163" t="inlineStr"/>
+      <c r="DE163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="n">
+        <v>90</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F164" s="1" t="n">
+        <v>46293.37589349537</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="n">
+        <v>0</v>
+      </c>
+      <c r="I164" t="n">
+        <v>0</v>
+      </c>
+      <c r="J164" t="n">
+        <v>0</v>
+      </c>
+      <c r="K164" t="n">
+        <v>0</v>
+      </c>
+      <c r="L164" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" t="n">
+        <v>0</v>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>주임 박상태</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr"/>
+      <c r="P164" t="n">
+        <v>90</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>4200</v>
+      </c>
+      <c r="R164" t="n">
+        <v>0</v>
+      </c>
+      <c r="S164" t="n">
+        <v>0</v>
+      </c>
+      <c r="T164" t="n">
+        <v>378000</v>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="V164" t="n">
+        <v>0</v>
+      </c>
+      <c r="W164" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X164" t="inlineStr"/>
+      <c r="Y164" t="inlineStr"/>
+      <c r="Z164" t="inlineStr"/>
+      <c r="AA164" t="inlineStr"/>
+      <c r="AB164" t="inlineStr"/>
+      <c r="AC164" t="inlineStr"/>
+      <c r="AD164" t="inlineStr"/>
+      <c r="AE164" t="inlineStr"/>
+      <c r="AF164" t="inlineStr"/>
+      <c r="AG164" t="inlineStr"/>
+      <c r="AH164" t="inlineStr"/>
+      <c r="AI164" t="inlineStr"/>
+      <c r="AJ164" t="inlineStr"/>
+      <c r="AK164" t="inlineStr"/>
+      <c r="AL164" t="inlineStr"/>
+      <c r="AM164" t="inlineStr"/>
+      <c r="AN164" t="inlineStr"/>
+      <c r="AO164" t="inlineStr"/>
+      <c r="AP164" t="inlineStr"/>
+      <c r="AQ164" t="inlineStr"/>
+      <c r="AR164" t="inlineStr"/>
+      <c r="AS164" t="inlineStr"/>
+      <c r="AT164" t="inlineStr"/>
+      <c r="AU164" t="inlineStr"/>
+      <c r="AV164" t="inlineStr"/>
+      <c r="AW164" t="inlineStr"/>
+      <c r="AX164" t="inlineStr"/>
+      <c r="AY164" t="inlineStr"/>
+      <c r="AZ164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG164" t="inlineStr">
+        <is>
+          <t>81루5100 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH164" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI164" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ164" t="inlineStr"/>
+      <c r="BK164" t="inlineStr"/>
+      <c r="BL164" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM164" t="inlineStr"/>
+      <c r="BN164" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO164" t="inlineStr"/>
+      <c r="BP164" t="inlineStr"/>
+      <c r="BQ164" t="inlineStr"/>
+      <c r="BR164" t="inlineStr"/>
+      <c r="BS164" t="inlineStr"/>
+      <c r="BT164" t="inlineStr"/>
+      <c r="BU164" t="inlineStr"/>
+      <c r="BV164" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW164" t="inlineStr"/>
+      <c r="BX164" t="inlineStr"/>
+      <c r="BY164" t="inlineStr"/>
+      <c r="BZ164" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA164" t="inlineStr"/>
+      <c r="CB164" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC164" t="inlineStr">
+        <is>
+          <t>250mm 초과 [10인치 이상] (1.0)</t>
+        </is>
+      </c>
+      <c r="CD164" t="inlineStr"/>
+      <c r="CE164" t="inlineStr"/>
+      <c r="CF164" t="inlineStr"/>
+      <c r="CG164" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH164" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI164" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ164" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK164" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL164" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM164" t="inlineStr"/>
+      <c r="CN164" t="inlineStr"/>
+      <c r="CO164" t="inlineStr"/>
+      <c r="CP164" t="inlineStr"/>
+      <c r="CQ164" t="inlineStr"/>
+      <c r="CR164" t="inlineStr"/>
+      <c r="CS164" t="inlineStr"/>
+      <c r="CT164" t="inlineStr"/>
+      <c r="CU164" t="inlineStr"/>
+      <c r="CV164" t="inlineStr"/>
+      <c r="CW164" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX164" t="inlineStr"/>
+      <c r="CY164" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ164" t="inlineStr"/>
+      <c r="DA164" t="inlineStr"/>
+      <c r="DB164" t="inlineStr"/>
+      <c r="DC164" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD164" t="inlineStr"/>
+      <c r="DE164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>410</v>
+      </c>
+      <c r="D165" t="n">
+        <v>30</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F165" s="1" t="n">
+        <v>46293.3813474074</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="n">
+        <v>0</v>
+      </c>
+      <c r="I165" t="n">
+        <v>0</v>
+      </c>
+      <c r="J165" t="n">
+        <v>0</v>
+      </c>
+      <c r="K165" t="n">
+        <v>0</v>
+      </c>
+      <c r="L165" t="n">
+        <v>0</v>
+      </c>
+      <c r="M165" t="n">
+        <v>0</v>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>주임 김성렬</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>R-ray(se-75)</t>
+        </is>
+      </c>
+      <c r="P165" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R165" t="n">
+        <v>0</v>
+      </c>
+      <c r="S165" t="n">
+        <v>0</v>
+      </c>
+      <c r="T165" t="n">
+        <v>765000</v>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V165" t="n">
+        <v>0</v>
+      </c>
+      <c r="W165" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="X165" t="inlineStr">
+        <is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="Y165" t="inlineStr">
+        <is>
+          <t>대리 우명광</t>
+        </is>
+      </c>
+      <c r="Z165" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="AA165" t="inlineStr">
+        <is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="AB165" t="inlineStr"/>
+      <c r="AC165" t="inlineStr"/>
+      <c r="AD165" t="inlineStr"/>
+      <c r="AE165" t="inlineStr"/>
+      <c r="AF165" t="inlineStr"/>
+      <c r="AG165" t="inlineStr"/>
+      <c r="AH165" t="inlineStr"/>
+      <c r="AI165" t="inlineStr"/>
+      <c r="AJ165" t="inlineStr"/>
+      <c r="AK165" t="inlineStr"/>
+      <c r="AL165" t="inlineStr"/>
+      <c r="AM165" t="inlineStr"/>
+      <c r="AN165" t="inlineStr"/>
+      <c r="AO165" t="inlineStr"/>
+      <c r="AP165" t="inlineStr"/>
+      <c r="AQ165" t="inlineStr"/>
+      <c r="AR165" t="inlineStr"/>
+      <c r="AS165" t="inlineStr"/>
+      <c r="AT165" t="inlineStr"/>
+      <c r="AU165" t="inlineStr"/>
+      <c r="AV165" t="inlineStr"/>
+      <c r="AW165" t="inlineStr"/>
+      <c r="AX165" t="inlineStr"/>
+      <c r="AY165" t="inlineStr"/>
+      <c r="AZ165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG165" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH165" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI165" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="BJ165" t="inlineStr"/>
+      <c r="BK165" t="inlineStr"/>
+      <c r="BL165" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM165" t="inlineStr"/>
+      <c r="BN165" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO165" t="inlineStr"/>
+      <c r="BP165" t="inlineStr"/>
+      <c r="BQ165" t="inlineStr"/>
+      <c r="BR165" t="inlineStr"/>
+      <c r="BS165" t="inlineStr"/>
+      <c r="BT165" t="inlineStr"/>
+      <c r="BU165" t="inlineStr"/>
+      <c r="BV165" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW165" t="inlineStr"/>
+      <c r="BX165" t="inlineStr"/>
+      <c r="BY165" t="inlineStr"/>
+      <c r="BZ165" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA165" t="inlineStr"/>
+      <c r="CB165" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC165" t="inlineStr">
+        <is>
+          <t>Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD165" t="inlineStr">
+        <is>
+          <t>조건없음 (1.0)</t>
+        </is>
+      </c>
+      <c r="CE165" t="inlineStr"/>
+      <c r="CF165" t="inlineStr"/>
+      <c r="CG165" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH165" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI165" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ165" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK165" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL165" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM165" t="inlineStr"/>
+      <c r="CN165" t="inlineStr"/>
+      <c r="CO165" t="inlineStr"/>
+      <c r="CP165" t="inlineStr"/>
+      <c r="CQ165" t="inlineStr"/>
+      <c r="CR165" t="inlineStr"/>
+      <c r="CS165" t="inlineStr"/>
+      <c r="CT165" t="inlineStr"/>
+      <c r="CU165" t="inlineStr"/>
+      <c r="CV165" t="inlineStr"/>
+      <c r="CW165" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX165" t="inlineStr"/>
+      <c r="CY165" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ165" t="inlineStr"/>
+      <c r="DA165" t="inlineStr">
+        <is>
+          <t>주배관</t>
+        </is>
+      </c>
+      <c r="DB165" t="inlineStr"/>
+      <c r="DC165" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD165" t="inlineStr"/>
+      <c r="DE165" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="n">
+        <v>46078</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="n">
+        <v>50</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F166" s="1" t="n">
+        <v>46293.38191709491</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" t="n">
+        <v>0</v>
+      </c>
+      <c r="I166" t="n">
+        <v>0</v>
+      </c>
+      <c r="J166" t="n">
+        <v>0</v>
+      </c>
+      <c r="K166" t="n">
+        <v>0</v>
+      </c>
+      <c r="L166" t="n">
+        <v>0</v>
+      </c>
+      <c r="M166" t="n">
+        <v>0</v>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>주임 박상태</t>
+        </is>
+      </c>
+      <c r="O166" t="inlineStr"/>
+      <c r="P166" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>4200</v>
+      </c>
+      <c r="R166" t="n">
+        <v>0</v>
+      </c>
+      <c r="S166" t="n">
+        <v>0</v>
+      </c>
+      <c r="T166" t="n">
+        <v>210000</v>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="V166" t="n">
+        <v>0</v>
+      </c>
+      <c r="W166" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X166" t="inlineStr"/>
+      <c r="Y166" t="inlineStr"/>
+      <c r="Z166" t="inlineStr"/>
+      <c r="AA166" t="inlineStr"/>
+      <c r="AB166" t="inlineStr"/>
+      <c r="AC166" t="inlineStr"/>
+      <c r="AD166" t="inlineStr"/>
+      <c r="AE166" t="inlineStr"/>
+      <c r="AF166" t="inlineStr"/>
+      <c r="AG166" t="inlineStr"/>
+      <c r="AH166" t="inlineStr"/>
+      <c r="AI166" t="inlineStr"/>
+      <c r="AJ166" t="inlineStr"/>
+      <c r="AK166" t="inlineStr"/>
+      <c r="AL166" t="inlineStr"/>
+      <c r="AM166" t="inlineStr"/>
+      <c r="AN166" t="inlineStr"/>
+      <c r="AO166" t="inlineStr"/>
+      <c r="AP166" t="inlineStr"/>
+      <c r="AQ166" t="inlineStr"/>
+      <c r="AR166" t="inlineStr"/>
+      <c r="AS166" t="inlineStr"/>
+      <c r="AT166" t="inlineStr"/>
+      <c r="AU166" t="inlineStr"/>
+      <c r="AV166" t="inlineStr"/>
+      <c r="AW166" t="inlineStr"/>
+      <c r="AX166" t="inlineStr"/>
+      <c r="AY166" t="inlineStr"/>
+      <c r="AZ166" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA166" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB166" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC166" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD166" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE166" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF166" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG166" t="inlineStr">
+        <is>
+          <t>81루5100 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH166" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI166" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ166" t="inlineStr"/>
+      <c r="BK166" t="inlineStr"/>
+      <c r="BL166" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM166" t="inlineStr"/>
+      <c r="BN166" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO166" t="inlineStr"/>
+      <c r="BP166" t="inlineStr"/>
+      <c r="BQ166" t="inlineStr"/>
+      <c r="BR166" t="inlineStr"/>
+      <c r="BS166" t="inlineStr"/>
+      <c r="BT166" t="inlineStr"/>
+      <c r="BU166" t="inlineStr"/>
+      <c r="BV166" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW166" t="inlineStr"/>
+      <c r="BX166" t="inlineStr"/>
+      <c r="BY166" t="inlineStr"/>
+      <c r="BZ166" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA166" t="inlineStr"/>
+      <c r="CB166" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC166" t="inlineStr">
+        <is>
+          <t>250mm 초과 [10인치 이상] (1.0)</t>
+        </is>
+      </c>
+      <c r="CD166" t="inlineStr"/>
+      <c r="CE166" t="inlineStr"/>
+      <c r="CF166" t="inlineStr"/>
+      <c r="CG166" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH166" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI166" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ166" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK166" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL166" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM166" t="inlineStr"/>
+      <c r="CN166" t="inlineStr"/>
+      <c r="CO166" t="inlineStr"/>
+      <c r="CP166" t="inlineStr"/>
+      <c r="CQ166" t="inlineStr"/>
+      <c r="CR166" t="inlineStr"/>
+      <c r="CS166" t="inlineStr"/>
+      <c r="CT166" t="inlineStr"/>
+      <c r="CU166" t="inlineStr"/>
+      <c r="CV166" t="inlineStr"/>
+      <c r="CW166" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX166" t="inlineStr"/>
+      <c r="CY166" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ166" t="inlineStr"/>
+      <c r="DA166" t="inlineStr"/>
+      <c r="DB166" t="inlineStr"/>
+      <c r="DC166" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD166" t="inlineStr"/>
+      <c r="DE166" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>410</v>
+      </c>
+      <c r="D167" t="n">
+        <v>44</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F167" s="1" t="n">
+        <v>46293.38564383102</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="n">
+        <v>0</v>
+      </c>
+      <c r="I167" t="n">
+        <v>0</v>
+      </c>
+      <c r="J167" t="n">
+        <v>0</v>
+      </c>
+      <c r="K167" t="n">
+        <v>0</v>
+      </c>
+      <c r="L167" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" t="n">
+        <v>0</v>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>주임 김성렬</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>R-ray(se-75)</t>
+        </is>
+      </c>
+      <c r="P167" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R167" t="n">
+        <v>0</v>
+      </c>
+      <c r="S167" t="n">
+        <v>0</v>
+      </c>
+      <c r="T167" t="n">
+        <v>1122000</v>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V167" t="n">
+        <v>0</v>
+      </c>
+      <c r="W167" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="Y167" t="inlineStr">
+        <is>
+          <t>대리 우명광</t>
+        </is>
+      </c>
+      <c r="Z167" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="AA167" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="AB167" t="inlineStr">
+        <is>
+          <t>계장 장승대</t>
+        </is>
+      </c>
+      <c r="AC167" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="AD167" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="AE167" t="inlineStr"/>
+      <c r="AF167" t="inlineStr"/>
+      <c r="AG167" t="inlineStr"/>
+      <c r="AH167" t="inlineStr"/>
+      <c r="AI167" t="inlineStr"/>
+      <c r="AJ167" t="inlineStr"/>
+      <c r="AK167" t="inlineStr"/>
+      <c r="AL167" t="inlineStr"/>
+      <c r="AM167" t="inlineStr"/>
+      <c r="AN167" t="inlineStr"/>
+      <c r="AO167" t="inlineStr"/>
+      <c r="AP167" t="inlineStr"/>
+      <c r="AQ167" t="inlineStr"/>
+      <c r="AR167" t="inlineStr"/>
+      <c r="AS167" t="inlineStr"/>
+      <c r="AT167" t="inlineStr"/>
+      <c r="AU167" t="inlineStr"/>
+      <c r="AV167" t="inlineStr"/>
+      <c r="AW167" t="inlineStr"/>
+      <c r="AX167" t="inlineStr"/>
+      <c r="AY167" t="inlineStr"/>
+      <c r="AZ167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG167" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스) || 90너4889 (탑차)</t>
+        </is>
+      </c>
+      <c r="BH167" t="inlineStr">
+        <is>
+          <t>40 || 40</t>
+        </is>
+      </c>
+      <c r="BI167" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ167" t="inlineStr">
+        <is>
+          <t>||</t>
+        </is>
+      </c>
+      <c r="BK167" t="inlineStr"/>
+      <c r="BL167" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM167" t="inlineStr"/>
+      <c r="BN167" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO167" t="inlineStr"/>
+      <c r="BP167" t="inlineStr"/>
+      <c r="BQ167" t="inlineStr"/>
+      <c r="BR167" t="inlineStr"/>
+      <c r="BS167" t="inlineStr"/>
+      <c r="BT167" t="inlineStr"/>
+      <c r="BU167" t="inlineStr"/>
+      <c r="BV167" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW167" t="inlineStr"/>
+      <c r="BX167" t="inlineStr"/>
+      <c r="BY167" t="inlineStr"/>
+      <c r="BZ167" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA167" t="inlineStr"/>
+      <c r="CB167" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC167" t="inlineStr">
+        <is>
+          <t>Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD167" t="inlineStr">
+        <is>
+          <t>조건없음 (1.0)</t>
+        </is>
+      </c>
+      <c r="CE167" t="inlineStr"/>
+      <c r="CF167" t="inlineStr"/>
+      <c r="CG167" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH167" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI167" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ167" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK167" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL167" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM167" t="inlineStr"/>
+      <c r="CN167" t="inlineStr"/>
+      <c r="CO167" t="inlineStr"/>
+      <c r="CP167" t="inlineStr"/>
+      <c r="CQ167" t="inlineStr"/>
+      <c r="CR167" t="inlineStr"/>
+      <c r="CS167" t="inlineStr"/>
+      <c r="CT167" t="inlineStr"/>
+      <c r="CU167" t="inlineStr"/>
+      <c r="CV167" t="inlineStr"/>
+      <c r="CW167" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX167" t="inlineStr"/>
+      <c r="CY167" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ167" t="inlineStr"/>
+      <c r="DA167" t="inlineStr">
+        <is>
+          <t>주배관</t>
+        </is>
+      </c>
+      <c r="DB167" t="inlineStr"/>
+      <c r="DC167" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD167" t="inlineStr"/>
+      <c r="DE167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+      <c r="D168" t="n">
+        <v>50</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F168" s="1" t="n">
+        <v>46293.38812679398</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="n">
+        <v>0</v>
+      </c>
+      <c r="I168" t="n">
+        <v>0</v>
+      </c>
+      <c r="J168" t="n">
+        <v>0</v>
+      </c>
+      <c r="K168" t="n">
+        <v>0</v>
+      </c>
+      <c r="L168" t="n">
+        <v>0</v>
+      </c>
+      <c r="M168" t="n">
+        <v>0</v>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O168" t="inlineStr"/>
+      <c r="P168" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>4200</v>
+      </c>
+      <c r="R168" t="n">
+        <v>0</v>
+      </c>
+      <c r="S168" t="n">
+        <v>0</v>
+      </c>
+      <c r="T168" t="n">
+        <v>210000</v>
+      </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="V168" t="n">
+        <v>0</v>
+      </c>
+      <c r="W168" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X168" t="inlineStr"/>
+      <c r="Y168" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="Z168" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA168" t="inlineStr"/>
+      <c r="AB168" t="inlineStr"/>
+      <c r="AC168" t="inlineStr"/>
+      <c r="AD168" t="inlineStr"/>
+      <c r="AE168" t="inlineStr"/>
+      <c r="AF168" t="inlineStr"/>
+      <c r="AG168" t="inlineStr"/>
+      <c r="AH168" t="inlineStr"/>
+      <c r="AI168" t="inlineStr"/>
+      <c r="AJ168" t="inlineStr"/>
+      <c r="AK168" t="inlineStr"/>
+      <c r="AL168" t="inlineStr"/>
+      <c r="AM168" t="inlineStr"/>
+      <c r="AN168" t="inlineStr"/>
+      <c r="AO168" t="inlineStr"/>
+      <c r="AP168" t="inlineStr"/>
+      <c r="AQ168" t="inlineStr"/>
+      <c r="AR168" t="inlineStr"/>
+      <c r="AS168" t="inlineStr"/>
+      <c r="AT168" t="inlineStr"/>
+      <c r="AU168" t="inlineStr"/>
+      <c r="AV168" t="inlineStr"/>
+      <c r="AW168" t="inlineStr"/>
+      <c r="AX168" t="inlineStr"/>
+      <c r="AY168" t="inlineStr"/>
+      <c r="AZ168" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA168" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB168" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC168" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD168" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE168" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF168" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG168" t="inlineStr">
+        <is>
+          <t>81루5100 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH168" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI168" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ168" t="inlineStr"/>
+      <c r="BK168" t="inlineStr"/>
+      <c r="BL168" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM168" t="inlineStr"/>
+      <c r="BN168" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO168" t="inlineStr"/>
+      <c r="BP168" t="inlineStr"/>
+      <c r="BQ168" t="inlineStr"/>
+      <c r="BR168" t="inlineStr"/>
+      <c r="BS168" t="inlineStr"/>
+      <c r="BT168" t="inlineStr"/>
+      <c r="BU168" t="inlineStr"/>
+      <c r="BV168" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW168" t="inlineStr"/>
+      <c r="BX168" t="inlineStr"/>
+      <c r="BY168" t="inlineStr"/>
+      <c r="BZ168" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA168" t="inlineStr"/>
+      <c r="CB168" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC168" t="inlineStr">
+        <is>
+          <t>250mm 초과 [10인치 이상] (1.0)</t>
+        </is>
+      </c>
+      <c r="CD168" t="inlineStr"/>
+      <c r="CE168" t="inlineStr"/>
+      <c r="CF168" t="inlineStr"/>
+      <c r="CG168" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH168" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI168" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ168" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK168" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL168" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM168" t="inlineStr"/>
+      <c r="CN168" t="inlineStr"/>
+      <c r="CO168" t="inlineStr"/>
+      <c r="CP168" t="inlineStr"/>
+      <c r="CQ168" t="inlineStr"/>
+      <c r="CR168" t="inlineStr"/>
+      <c r="CS168" t="inlineStr"/>
+      <c r="CT168" t="inlineStr"/>
+      <c r="CU168" t="inlineStr"/>
+      <c r="CV168" t="inlineStr"/>
+      <c r="CW168" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX168" t="inlineStr"/>
+      <c r="CY168" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ168" t="inlineStr"/>
+      <c r="DA168" t="inlineStr"/>
+      <c r="DB168" t="inlineStr"/>
+      <c r="DC168" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD168" t="inlineStr"/>
+      <c r="DE168" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>0</v>
+      </c>
+      <c r="D169" t="n">
+        <v>10</v>
+      </c>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" s="1" t="n">
+        <v>46293.39197844582</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="n">
+        <v>0</v>
+      </c>
+      <c r="I169" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" t="n">
+        <v>0</v>
+      </c>
+      <c r="K169" t="n">
+        <v>0</v>
+      </c>
+      <c r="L169" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" t="n">
+        <v>0</v>
+      </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O169" t="inlineStr"/>
+      <c r="P169" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>14300</v>
+      </c>
+      <c r="R169" t="n">
+        <v>0</v>
+      </c>
+      <c r="S169" t="n">
+        <v>0</v>
+      </c>
+      <c r="T169" t="n">
+        <v>143000</v>
+      </c>
+      <c r="U169" t="inlineStr">
+        <is>
+          <t>PMI</t>
+        </is>
+      </c>
+      <c r="V169" t="n">
+        <v>0</v>
+      </c>
+      <c r="W169" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X169" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y169" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="Z169" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB169" t="inlineStr"/>
+      <c r="AC169" t="inlineStr"/>
+      <c r="AD169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE169" t="inlineStr"/>
+      <c r="AF169" t="inlineStr"/>
+      <c r="AG169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH169" t="inlineStr"/>
+      <c r="AI169" t="inlineStr"/>
+      <c r="AJ169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK169" t="inlineStr"/>
+      <c r="AL169" t="inlineStr"/>
+      <c r="AM169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN169" t="inlineStr"/>
+      <c r="AO169" t="inlineStr"/>
+      <c r="AP169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ169" t="inlineStr"/>
+      <c r="AR169" t="inlineStr"/>
+      <c r="AS169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT169" t="inlineStr"/>
+      <c r="AU169" t="inlineStr"/>
+      <c r="AV169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW169" t="inlineStr"/>
+      <c r="AX169" t="inlineStr"/>
+      <c r="AY169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG169" t="inlineStr"/>
+      <c r="BH169" t="inlineStr"/>
+      <c r="BI169" t="inlineStr"/>
+      <c r="BJ169" t="inlineStr"/>
+      <c r="BK169" t="inlineStr"/>
+      <c r="BL169" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM169" t="inlineStr"/>
+      <c r="BN169" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO169" t="inlineStr"/>
+      <c r="BP169" t="inlineStr"/>
+      <c r="BQ169" t="inlineStr"/>
+      <c r="BR169" t="inlineStr"/>
+      <c r="BS169" t="inlineStr"/>
+      <c r="BT169" t="inlineStr"/>
+      <c r="BU169" t="inlineStr"/>
+      <c r="BV169" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW169" t="inlineStr"/>
+      <c r="BX169" t="inlineStr"/>
+      <c r="BY169" t="inlineStr"/>
+      <c r="BZ169" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA169" t="inlineStr"/>
+      <c r="CB169" t="inlineStr"/>
+      <c r="CC169" t="inlineStr"/>
+      <c r="CD169" t="inlineStr"/>
+      <c r="CE169" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF169" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG169" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH169" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI169" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ169" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK169" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL169" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM169" t="inlineStr"/>
+      <c r="CN169" t="inlineStr"/>
+      <c r="CO169" t="inlineStr"/>
+      <c r="CP169" t="inlineStr"/>
+      <c r="CQ169" t="inlineStr"/>
+      <c r="CR169" t="inlineStr"/>
+      <c r="CS169" t="inlineStr"/>
+      <c r="CT169" t="inlineStr"/>
+      <c r="CU169" t="inlineStr"/>
+      <c r="CV169" t="inlineStr"/>
+      <c r="CW169" t="inlineStr"/>
+      <c r="CX169" t="inlineStr"/>
+      <c r="CY169" t="inlineStr"/>
+      <c r="CZ169" t="inlineStr"/>
+      <c r="DA169" t="inlineStr"/>
+      <c r="DB169" t="inlineStr"/>
+      <c r="DC169" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD169" t="inlineStr"/>
+      <c r="DE169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr"/>
+      <c r="D170" t="n">
+        <v>70</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F170" s="1" t="n">
+        <v>46293.40617878191</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="n">
+        <v>0</v>
+      </c>
+      <c r="I170" t="n">
+        <v>0</v>
+      </c>
+      <c r="J170" t="n">
+        <v>0</v>
+      </c>
+      <c r="K170" t="n">
+        <v>0</v>
+      </c>
+      <c r="L170" t="n">
+        <v>0</v>
+      </c>
+      <c r="M170" t="n">
+        <v>0</v>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr"/>
+      <c r="P170" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>4200</v>
+      </c>
+      <c r="R170" t="n">
+        <v>0</v>
+      </c>
+      <c r="S170" t="n">
+        <v>0</v>
+      </c>
+      <c r="T170" t="n">
+        <v>294000</v>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="V170" t="n">
+        <v>0</v>
+      </c>
+      <c r="W170" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X170" t="inlineStr"/>
+      <c r="Y170" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="Z170" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA170" t="inlineStr"/>
+      <c r="AB170" t="inlineStr"/>
+      <c r="AC170" t="inlineStr"/>
+      <c r="AD170" t="inlineStr"/>
+      <c r="AE170" t="inlineStr"/>
+      <c r="AF170" t="inlineStr"/>
+      <c r="AG170" t="inlineStr"/>
+      <c r="AH170" t="inlineStr"/>
+      <c r="AI170" t="inlineStr"/>
+      <c r="AJ170" t="inlineStr"/>
+      <c r="AK170" t="inlineStr"/>
+      <c r="AL170" t="inlineStr"/>
+      <c r="AM170" t="inlineStr"/>
+      <c r="AN170" t="inlineStr"/>
+      <c r="AO170" t="inlineStr"/>
+      <c r="AP170" t="inlineStr"/>
+      <c r="AQ170" t="inlineStr"/>
+      <c r="AR170" t="inlineStr"/>
+      <c r="AS170" t="inlineStr"/>
+      <c r="AT170" t="inlineStr"/>
+      <c r="AU170" t="inlineStr"/>
+      <c r="AV170" t="inlineStr"/>
+      <c r="AW170" t="inlineStr"/>
+      <c r="AX170" t="inlineStr"/>
+      <c r="AY170" t="inlineStr"/>
+      <c r="AZ170" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA170" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB170" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC170" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD170" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE170" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF170" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG170" t="inlineStr">
+        <is>
+          <t>81루5100 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH170" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI170" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ170" t="inlineStr"/>
+      <c r="BK170" t="inlineStr"/>
+      <c r="BL170" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM170" t="inlineStr"/>
+      <c r="BN170" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO170" t="inlineStr"/>
+      <c r="BP170" t="inlineStr"/>
+      <c r="BQ170" t="inlineStr"/>
+      <c r="BR170" t="inlineStr"/>
+      <c r="BS170" t="inlineStr"/>
+      <c r="BT170" t="inlineStr"/>
+      <c r="BU170" t="inlineStr"/>
+      <c r="BV170" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW170" t="inlineStr"/>
+      <c r="BX170" t="inlineStr"/>
+      <c r="BY170" t="inlineStr"/>
+      <c r="BZ170" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA170" t="inlineStr"/>
+      <c r="CB170" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC170" t="inlineStr">
+        <is>
+          <t>250mm 초과 [10인치 이상] (1.0)</t>
+        </is>
+      </c>
+      <c r="CD170" t="inlineStr"/>
+      <c r="CE170" t="inlineStr"/>
+      <c r="CF170" t="inlineStr"/>
+      <c r="CG170" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH170" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI170" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ170" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK170" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL170" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM170" t="inlineStr"/>
+      <c r="CN170" t="inlineStr"/>
+      <c r="CO170" t="inlineStr"/>
+      <c r="CP170" t="inlineStr"/>
+      <c r="CQ170" t="inlineStr"/>
+      <c r="CR170" t="inlineStr"/>
+      <c r="CS170" t="inlineStr"/>
+      <c r="CT170" t="inlineStr"/>
+      <c r="CU170" t="inlineStr"/>
+      <c r="CV170" t="inlineStr"/>
+      <c r="CW170" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX170" t="inlineStr"/>
+      <c r="CY170" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="CZ170" t="inlineStr"/>
+      <c r="DA170" t="inlineStr"/>
+      <c r="DB170" t="inlineStr"/>
+      <c r="DC170" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD170" t="inlineStr"/>
+      <c r="DE170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>46080</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>410</v>
+      </c>
+      <c r="D171" t="n">
+        <v>18</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F171" s="1" t="n">
+        <v>46293.40807263476</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="n">
+        <v>0</v>
+      </c>
+      <c r="I171" t="n">
+        <v>0</v>
+      </c>
+      <c r="J171" t="n">
+        <v>0</v>
+      </c>
+      <c r="K171" t="n">
+        <v>0</v>
+      </c>
+      <c r="L171" t="n">
+        <v>0</v>
+      </c>
+      <c r="M171" t="n">
+        <v>0</v>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>주임 김성렬</t>
+        </is>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>R-ray(se-75)</t>
+        </is>
+      </c>
+      <c r="P171" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R171" t="n">
+        <v>0</v>
+      </c>
+      <c r="S171" t="n">
+        <v>0</v>
+      </c>
+      <c r="T171" t="n">
+        <v>459000</v>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V171" t="n">
+        <v>0</v>
+      </c>
+      <c r="W171" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="X171" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="Y171" t="inlineStr">
+        <is>
+          <t>대리 우명광</t>
+        </is>
+      </c>
+      <c r="Z171" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="AA171" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="AB171" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="AC171" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="AD171" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
+      </c>
+      <c r="AE171" t="inlineStr"/>
+      <c r="AF171" t="inlineStr"/>
+      <c r="AG171" t="inlineStr"/>
+      <c r="AH171" t="inlineStr"/>
+      <c r="AI171" t="inlineStr"/>
+      <c r="AJ171" t="inlineStr"/>
+      <c r="AK171" t="inlineStr"/>
+      <c r="AL171" t="inlineStr"/>
+      <c r="AM171" t="inlineStr"/>
+      <c r="AN171" t="inlineStr"/>
+      <c r="AO171" t="inlineStr"/>
+      <c r="AP171" t="inlineStr"/>
+      <c r="AQ171" t="inlineStr"/>
+      <c r="AR171" t="inlineStr"/>
+      <c r="AS171" t="inlineStr"/>
+      <c r="AT171" t="inlineStr"/>
+      <c r="AU171" t="inlineStr"/>
+      <c r="AV171" t="inlineStr"/>
+      <c r="AW171" t="inlineStr"/>
+      <c r="AX171" t="inlineStr"/>
+      <c r="AY171" t="inlineStr"/>
+      <c r="AZ171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG171" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH171" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI171" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금</t>
+        </is>
+      </c>
+      <c r="BJ171" t="inlineStr"/>
+      <c r="BK171" t="inlineStr"/>
+      <c r="BL171" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM171" t="inlineStr"/>
+      <c r="BN171" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO171" t="inlineStr"/>
+      <c r="BP171" t="inlineStr"/>
+      <c r="BQ171" t="inlineStr"/>
+      <c r="BR171" t="inlineStr"/>
+      <c r="BS171" t="inlineStr"/>
+      <c r="BT171" t="inlineStr"/>
+      <c r="BU171" t="inlineStr"/>
+      <c r="BV171" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW171" t="inlineStr"/>
+      <c r="BX171" t="inlineStr"/>
+      <c r="BY171" t="inlineStr"/>
+      <c r="BZ171" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA171" t="inlineStr"/>
+      <c r="CB171" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC171" t="inlineStr">
+        <is>
+          <t>Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD171" t="inlineStr">
+        <is>
+          <t>조건없음 (1.0)</t>
+        </is>
+      </c>
+      <c r="CE171" t="inlineStr"/>
+      <c r="CF171" t="inlineStr"/>
+      <c r="CG171" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH171" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI171" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ171" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK171" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL171" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM171" t="inlineStr"/>
+      <c r="CN171" t="inlineStr"/>
+      <c r="CO171" t="inlineStr"/>
+      <c r="CP171" t="inlineStr"/>
+      <c r="CQ171" t="inlineStr"/>
+      <c r="CR171" t="inlineStr"/>
+      <c r="CS171" t="inlineStr"/>
+      <c r="CT171" t="inlineStr"/>
+      <c r="CU171" t="inlineStr"/>
+      <c r="CV171" t="inlineStr"/>
+      <c r="CW171" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX171" t="inlineStr"/>
+      <c r="CY171" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="CZ171" t="inlineStr"/>
+      <c r="DA171" t="inlineStr">
+        <is>
+          <t>주배관</t>
+        </is>
+      </c>
+      <c r="DB171" t="inlineStr"/>
+      <c r="DC171" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD171" t="inlineStr"/>
+      <c r="DE171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
+        <v>46112</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr"/>
+      <c r="D172" t="n">
+        <v>100</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F172" s="1" t="n">
+        <v>46293.43436331792</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="n">
+        <v>0</v>
+      </c>
+      <c r="I172" t="n">
+        <v>0</v>
+      </c>
+      <c r="J172" t="n">
+        <v>0</v>
+      </c>
+      <c r="K172" t="n">
+        <v>0</v>
+      </c>
+      <c r="L172" t="n">
+        <v>0</v>
+      </c>
+      <c r="M172" t="n">
+        <v>0</v>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>주임 김진환</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr"/>
+      <c r="P172" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>4200</v>
+      </c>
+      <c r="R172" t="n">
+        <v>0</v>
+      </c>
+      <c r="S172" t="n">
+        <v>0</v>
+      </c>
+      <c r="T172" t="n">
+        <v>420000</v>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>PT</t>
+        </is>
+      </c>
+      <c r="V172" t="n">
+        <v>0</v>
+      </c>
+      <c r="W172" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~22:00</t>
+        </is>
+      </c>
+      <c r="X172" t="inlineStr">
+        <is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="Y172" t="inlineStr"/>
+      <c r="Z172" t="inlineStr"/>
+      <c r="AA172" t="inlineStr"/>
+      <c r="AB172" t="inlineStr"/>
+      <c r="AC172" t="inlineStr"/>
+      <c r="AD172" t="inlineStr"/>
+      <c r="AE172" t="inlineStr"/>
+      <c r="AF172" t="inlineStr"/>
+      <c r="AG172" t="inlineStr"/>
+      <c r="AH172" t="inlineStr"/>
+      <c r="AI172" t="inlineStr"/>
+      <c r="AJ172" t="inlineStr"/>
+      <c r="AK172" t="inlineStr"/>
+      <c r="AL172" t="inlineStr"/>
+      <c r="AM172" t="inlineStr"/>
+      <c r="AN172" t="inlineStr"/>
+      <c r="AO172" t="inlineStr"/>
+      <c r="AP172" t="inlineStr"/>
+      <c r="AQ172" t="inlineStr"/>
+      <c r="AR172" t="inlineStr"/>
+      <c r="AS172" t="inlineStr"/>
+      <c r="AT172" t="inlineStr"/>
+      <c r="AU172" t="inlineStr"/>
+      <c r="AV172" t="inlineStr"/>
+      <c r="AW172" t="inlineStr"/>
+      <c r="AX172" t="inlineStr"/>
+      <c r="AY172" t="inlineStr"/>
+      <c r="AZ172" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA172" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB172" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC172" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD172" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE172" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF172" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG172" t="inlineStr">
+        <is>
+          <t>90너4889 (탑차)</t>
+        </is>
+      </c>
+      <c r="BH172" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="BI172" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ172" t="inlineStr"/>
+      <c r="BK172" t="inlineStr"/>
+      <c r="BL172" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM172" t="inlineStr"/>
+      <c r="BN172" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO172" t="inlineStr"/>
+      <c r="BP172" t="inlineStr"/>
+      <c r="BQ172" t="inlineStr"/>
+      <c r="BR172" t="inlineStr"/>
+      <c r="BS172" t="inlineStr"/>
+      <c r="BT172" t="inlineStr"/>
+      <c r="BU172" t="inlineStr"/>
+      <c r="BV172" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW172" t="inlineStr"/>
+      <c r="BX172" t="inlineStr"/>
+      <c r="BY172" t="inlineStr"/>
+      <c r="BZ172" t="inlineStr">
+        <is>
+          <t>I/D</t>
+        </is>
+      </c>
+      <c r="CA172" t="inlineStr"/>
+      <c r="CB172" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC172" t="inlineStr">
+        <is>
+          <t>250mm 초과 [10인치 이상] (1.0)</t>
+        </is>
+      </c>
+      <c r="CD172" t="inlineStr"/>
+      <c r="CE172" t="inlineStr"/>
+      <c r="CF172" t="inlineStr"/>
+      <c r="CG172" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH172" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI172" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ172" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK172" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL172" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM172" t="inlineStr"/>
+      <c r="CN172" t="inlineStr"/>
+      <c r="CO172" t="inlineStr"/>
+      <c r="CP172" t="inlineStr"/>
+      <c r="CQ172" t="inlineStr"/>
+      <c r="CR172" t="inlineStr"/>
+      <c r="CS172" t="inlineStr"/>
+      <c r="CT172" t="inlineStr"/>
+      <c r="CU172" t="inlineStr"/>
+      <c r="CV172" t="inlineStr"/>
+      <c r="CW172" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX172" t="inlineStr"/>
+      <c r="CY172" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="CZ172" t="inlineStr"/>
+      <c r="DA172" t="inlineStr"/>
+      <c r="DB172" t="inlineStr"/>
+      <c r="DC172" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD172" t="inlineStr"/>
+      <c r="DE172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>K1 PJT</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>410</v>
+      </c>
+      <c r="D173" t="n">
+        <v>15</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="F173" s="1" t="n">
+        <v>46293.46815471132</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="n">
+        <v>0</v>
+      </c>
+      <c r="I173" t="n">
+        <v>0</v>
+      </c>
+      <c r="J173" t="n">
+        <v>0</v>
+      </c>
+      <c r="K173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L173" t="n">
+        <v>0</v>
+      </c>
+      <c r="M173" t="n">
+        <v>0</v>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>대리 김성현</t>
+        </is>
+      </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>R-ray(se-75)</t>
+        </is>
+      </c>
+      <c r="P173" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>25500</v>
+      </c>
+      <c r="R173" t="n">
+        <v>0</v>
+      </c>
+      <c r="S173" t="n">
+        <v>0</v>
+      </c>
+      <c r="T173" t="n">
+        <v>382500</v>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V173" t="n">
+        <v>0</v>
+      </c>
+      <c r="W173" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="X173" t="inlineStr">
+        <is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="Y173" t="inlineStr">
+        <is>
+          <t>주임 김성렬</t>
+        </is>
+      </c>
+      <c r="Z173" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="AA173" t="inlineStr">
+        <is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="AB173" t="inlineStr">
+        <is>
+          <t>주임 이경재</t>
+        </is>
+      </c>
+      <c r="AC173" t="inlineStr">
+        <is>
+          <t>(야간) 22:00~익일02:00</t>
+        </is>
+      </c>
+      <c r="AD173" t="inlineStr">
+        <is>
+          <t>20,000</t>
+        </is>
+      </c>
+      <c r="AE173" t="inlineStr"/>
+      <c r="AF173" t="inlineStr"/>
+      <c r="AG173" t="inlineStr"/>
+      <c r="AH173" t="inlineStr"/>
+      <c r="AI173" t="inlineStr"/>
+      <c r="AJ173" t="inlineStr"/>
+      <c r="AK173" t="inlineStr"/>
+      <c r="AL173" t="inlineStr"/>
+      <c r="AM173" t="inlineStr"/>
+      <c r="AN173" t="inlineStr"/>
+      <c r="AO173" t="inlineStr"/>
+      <c r="AP173" t="inlineStr"/>
+      <c r="AQ173" t="inlineStr"/>
+      <c r="AR173" t="inlineStr"/>
+      <c r="AS173" t="inlineStr"/>
+      <c r="AT173" t="inlineStr"/>
+      <c r="AU173" t="inlineStr"/>
+      <c r="AV173" t="inlineStr"/>
+      <c r="AW173" t="inlineStr"/>
+      <c r="AX173" t="inlineStr"/>
+      <c r="AY173" t="inlineStr"/>
+      <c r="AZ173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG173" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스) || 90너4889 (탑차)</t>
+        </is>
+      </c>
+      <c r="BH173" t="inlineStr">
+        <is>
+          <t>40 || 40</t>
+        </is>
+      </c>
+      <c r="BI173" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:잠금|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:잠금 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ173" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> || </t>
+        </is>
+      </c>
+      <c r="BK173" t="inlineStr"/>
+      <c r="BL173" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM173" t="inlineStr"/>
+      <c r="BN173" t="inlineStr">
+        <is>
+          <t>롯데건설</t>
+        </is>
+      </c>
+      <c r="BO173" t="inlineStr"/>
+      <c r="BP173" t="inlineStr"/>
+      <c r="BQ173" t="inlineStr"/>
+      <c r="BR173" t="inlineStr"/>
+      <c r="BS173" t="inlineStr"/>
+      <c r="BT173" t="inlineStr"/>
+      <c r="BU173" t="inlineStr"/>
+      <c r="BV173" t="inlineStr">
+        <is>
+          <t>pipe</t>
+        </is>
+      </c>
+      <c r="BW173" t="inlineStr"/>
+      <c r="BX173" t="inlineStr"/>
+      <c r="BY173" t="inlineStr"/>
+      <c r="BZ173" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA173" t="inlineStr"/>
+      <c r="CB173" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC173" t="inlineStr">
+        <is>
+          <t>Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD173" t="inlineStr">
+        <is>
+          <t>조건없음 (1.0)</t>
+        </is>
+      </c>
+      <c r="CE173" t="inlineStr"/>
+      <c r="CF173" t="inlineStr"/>
+      <c r="CG173" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH173" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI173" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ173" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK173" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL173" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM173" t="inlineStr"/>
+      <c r="CN173" t="inlineStr"/>
+      <c r="CO173" t="inlineStr"/>
+      <c r="CP173" t="inlineStr"/>
+      <c r="CQ173" t="inlineStr"/>
+      <c r="CR173" t="inlineStr"/>
+      <c r="CS173" t="inlineStr"/>
+      <c r="CT173" t="inlineStr"/>
+      <c r="CU173" t="inlineStr"/>
+      <c r="CV173" t="inlineStr"/>
+      <c r="CW173" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX173" t="inlineStr"/>
+      <c r="CY173" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="CZ173" t="inlineStr"/>
+      <c r="DA173" t="inlineStr">
+        <is>
+          <t>주배관</t>
+        </is>
+      </c>
+      <c r="DB173" t="inlineStr"/>
+      <c r="DC173" t="inlineStr">
+        <is>
+          <t>[당일 불량(REJ) 0.0개 발생]</t>
+        </is>
+      </c>
+      <c r="DD173" t="inlineStr"/>
+      <c r="DE173" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>